<commit_message>
New Treg manuscript figure variants
Also removed duplicate figures, data files, and pinned R to 4.3
</commit_message>
<xml_diff>
--- a/data/input/CD4_Treg_geneLists.xlsx
+++ b/data/input/CD4_Treg_geneLists.xlsx
@@ -1,19 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tedwards/Documents/projects/P589-1_Cerosaletti_Chen_foreign_autoreactive_CD4_Tcell_10X/data/input/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D433B7D-4DBF-5349-84B2-32B15F657555}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9600" yWindow="-23940" windowWidth="25760" windowHeight="18460" xr2:uid="{22A6F945-93EC-4C4C-8699-B7991E014781}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="curatedGrouped" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="154">
   <si>
     <t>CCR7</t>
   </si>
@@ -288,13 +282,224 @@
   </si>
   <si>
     <t>curated</t>
+  </si>
+  <si>
+    <t>Hollbacher</t>
+  </si>
+  <si>
+    <t>CSF2RB</t>
+  </si>
+  <si>
+    <t>HPGD</t>
+  </si>
+  <si>
+    <t>ICA1</t>
+  </si>
+  <si>
+    <t>IL1R1</t>
+  </si>
+  <si>
+    <t>IL1R2</t>
+  </si>
+  <si>
+    <t>METTL7A</t>
+  </si>
+  <si>
+    <t>RBMS3</t>
+  </si>
+  <si>
+    <t>SGMS1</t>
+  </si>
+  <si>
+    <t>STAM</t>
+  </si>
+  <si>
+    <t>TNFRSF1B</t>
+  </si>
+  <si>
+    <t>TRIB1</t>
+  </si>
+  <si>
+    <t>VAV3</t>
+  </si>
+  <si>
+    <t>VOPP1</t>
+  </si>
+  <si>
+    <t>ZBTB38</t>
+  </si>
+  <si>
+    <t>ZC2HC1A</t>
+  </si>
+  <si>
+    <t>ZNF532</t>
+  </si>
+  <si>
+    <t xml:space="preserve">category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gene</t>
+  </si>
+  <si>
+    <t xml:space="preserve">order</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Activation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CD40LG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TNFRSF9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CD69</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CD44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Naive</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TCF7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LEF1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Memory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CD27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CCR7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SELL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CD38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IL7R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Treg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FOXP3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IKZF2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IL2RA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BATF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LRRC32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ENTPD1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CTLA4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TIGIT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HLA-DRB1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Th subsets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CCR4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CCR6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CXCR3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CXCR5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PDCD1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GATA3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TBX21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RORA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RORC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BATF3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BCL6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Function</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BHLHE40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IL2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TNF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CSF2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IFNG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TGFB1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IL10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LAG3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HAVCR2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GZMB</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="5">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -316,6 +521,7 @@
     </font>
     <font>
       <sz val="11"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -687,14 +893,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8A4F54A-1648-B847-A1B7-47797666AE78}">
-  <dimension ref="A1:H29"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="15.5" customWidth="1"/>
+    <col min="1" max="1" width="15.5" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -719,8 +925,11 @@
       <c r="H1" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -745,8 +954,11 @@
       <c r="H2" s="4" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I2" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -771,8 +983,11 @@
       <c r="H3" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I3" s="4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4">
       <c r="A4" t="s">
         <v>50</v>
       </c>
@@ -797,8 +1012,11 @@
       <c r="H4" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I4" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5">
       <c r="A5" t="s">
         <v>51</v>
       </c>
@@ -823,8 +1041,11 @@
       <c r="H5" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I5" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="6">
       <c r="A6" t="s">
         <v>52</v>
       </c>
@@ -849,8 +1070,11 @@
       <c r="H6" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I6" s="4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="7">
       <c r="B7" t="s">
         <v>56</v>
       </c>
@@ -869,8 +1093,11 @@
       <c r="H7" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I7" s="4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="8">
       <c r="B8" t="s">
         <v>6</v>
       </c>
@@ -889,8 +1116,11 @@
       <c r="H8" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I8" s="4" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="9">
       <c r="B9" t="s">
         <v>7</v>
       </c>
@@ -909,8 +1139,11 @@
       <c r="H9" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I9" s="4" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="10">
       <c r="B10" t="s">
         <v>8</v>
       </c>
@@ -926,8 +1159,11 @@
       <c r="H10" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I10" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="11">
       <c r="B11" t="s">
         <v>9</v>
       </c>
@@ -943,8 +1179,11 @@
       <c r="H11" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I11" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="12">
       <c r="B12" t="s">
         <v>10</v>
       </c>
@@ -960,8 +1199,11 @@
       <c r="H12" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I12" s="4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="13">
       <c r="B13" t="s">
         <v>11</v>
       </c>
@@ -977,8 +1219,11 @@
       <c r="H13" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I13" s="4" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="14">
       <c r="B14" t="s">
         <v>12</v>
       </c>
@@ -991,72 +1236,99 @@
       <c r="H14" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I14" s="4" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="15">
       <c r="B15" t="s">
         <v>13</v>
       </c>
       <c r="H15" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I15" s="4" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="16">
       <c r="B16" t="s">
         <v>14</v>
       </c>
       <c r="H16" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="I16" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="17">
       <c r="B17" t="s">
         <v>15</v>
       </c>
       <c r="H17" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="I17" s="4" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="18">
       <c r="B18" t="s">
         <v>16</v>
       </c>
       <c r="H18" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="I18" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="19">
       <c r="B19" t="s">
         <v>17</v>
       </c>
       <c r="H19" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="I19" s="4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="20">
       <c r="B20" t="s">
         <v>57</v>
       </c>
       <c r="H20" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="I20" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="21">
       <c r="B21" t="s">
         <v>18</v>
       </c>
       <c r="H21" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="I21" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="22">
       <c r="B22" t="s">
         <v>19</v>
       </c>
       <c r="H22" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="I22" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="23">
       <c r="B23" t="s">
         <v>20</v>
       </c>
@@ -1064,7 +1336,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="24">
       <c r="B24" t="s">
         <v>21</v>
       </c>
@@ -1072,7 +1344,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="25">
       <c r="B25" t="s">
         <v>22</v>
       </c>
@@ -1080,27 +1352,534 @@
         <v>28</v>
       </c>
     </row>
-    <row r="26" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="26">
       <c r="H26" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="27">
       <c r="H27" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="28">
       <c r="H28" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="29" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="29">
       <c r="H29" t="s">
         <v>68</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B4" t="s">
+        <v>107</v>
+      </c>
+      <c r="C4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>104</v>
+      </c>
+      <c r="B5" t="s">
+        <v>108</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>109</v>
+      </c>
+      <c r="B6" t="s">
+        <v>110</v>
+      </c>
+      <c r="C6" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>109</v>
+      </c>
+      <c r="B7" t="s">
+        <v>111</v>
+      </c>
+      <c r="C7" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>112</v>
+      </c>
+      <c r="B8" t="s">
+        <v>113</v>
+      </c>
+      <c r="C8" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>112</v>
+      </c>
+      <c r="B9" t="s">
+        <v>114</v>
+      </c>
+      <c r="C9" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>112</v>
+      </c>
+      <c r="B10" t="s">
+        <v>115</v>
+      </c>
+      <c r="C10" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>112</v>
+      </c>
+      <c r="B11" t="s">
+        <v>116</v>
+      </c>
+      <c r="C11" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>112</v>
+      </c>
+      <c r="B12" t="s">
+        <v>117</v>
+      </c>
+      <c r="C12" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>112</v>
+      </c>
+      <c r="B13" t="s">
+        <v>118</v>
+      </c>
+      <c r="C13" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>112</v>
+      </c>
+      <c r="B14" t="s">
+        <v>119</v>
+      </c>
+      <c r="C14" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>120</v>
+      </c>
+      <c r="B15" t="s">
+        <v>121</v>
+      </c>
+      <c r="C15" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>120</v>
+      </c>
+      <c r="B16" t="s">
+        <v>122</v>
+      </c>
+      <c r="C16" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>120</v>
+      </c>
+      <c r="B17" t="s">
+        <v>123</v>
+      </c>
+      <c r="C17" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>120</v>
+      </c>
+      <c r="B18" t="s">
+        <v>124</v>
+      </c>
+      <c r="C18" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>120</v>
+      </c>
+      <c r="B19" t="s">
+        <v>125</v>
+      </c>
+      <c r="C19" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>120</v>
+      </c>
+      <c r="B20" t="s">
+        <v>126</v>
+      </c>
+      <c r="C20" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>120</v>
+      </c>
+      <c r="B21" t="s">
+        <v>127</v>
+      </c>
+      <c r="C21" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>120</v>
+      </c>
+      <c r="B22" t="s">
+        <v>128</v>
+      </c>
+      <c r="C22" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>120</v>
+      </c>
+      <c r="B23" t="s">
+        <v>129</v>
+      </c>
+      <c r="C23" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>130</v>
+      </c>
+      <c r="B24" t="s">
+        <v>131</v>
+      </c>
+      <c r="C24" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>130</v>
+      </c>
+      <c r="B25" t="s">
+        <v>132</v>
+      </c>
+      <c r="C25" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>130</v>
+      </c>
+      <c r="B26" t="s">
+        <v>133</v>
+      </c>
+      <c r="C26" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>130</v>
+      </c>
+      <c r="B27" t="s">
+        <v>134</v>
+      </c>
+      <c r="C27" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>130</v>
+      </c>
+      <c r="B28" t="s">
+        <v>135</v>
+      </c>
+      <c r="C28" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>130</v>
+      </c>
+      <c r="B29" t="s">
+        <v>136</v>
+      </c>
+      <c r="C29" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>130</v>
+      </c>
+      <c r="B30" t="s">
+        <v>137</v>
+      </c>
+      <c r="C30" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>130</v>
+      </c>
+      <c r="B31" t="s">
+        <v>138</v>
+      </c>
+      <c r="C31" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>130</v>
+      </c>
+      <c r="B32" t="s">
+        <v>139</v>
+      </c>
+      <c r="C32" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>130</v>
+      </c>
+      <c r="B33" t="s">
+        <v>140</v>
+      </c>
+      <c r="C33" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>130</v>
+      </c>
+      <c r="B34" t="s">
+        <v>141</v>
+      </c>
+      <c r="C34" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>142</v>
+      </c>
+      <c r="B35" t="s">
+        <v>143</v>
+      </c>
+      <c r="C35" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>142</v>
+      </c>
+      <c r="B36" t="s">
+        <v>144</v>
+      </c>
+      <c r="C36" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>142</v>
+      </c>
+      <c r="B37" t="s">
+        <v>145</v>
+      </c>
+      <c r="C37" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>142</v>
+      </c>
+      <c r="B38" t="s">
+        <v>146</v>
+      </c>
+      <c r="C38" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>142</v>
+      </c>
+      <c r="B39" t="s">
+        <v>147</v>
+      </c>
+      <c r="C39" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>142</v>
+      </c>
+      <c r="B40" t="s">
+        <v>148</v>
+      </c>
+      <c r="C40" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s">
+        <v>142</v>
+      </c>
+      <c r="B41" t="s">
+        <v>149</v>
+      </c>
+      <c r="C41" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>142</v>
+      </c>
+      <c r="B42" t="s">
+        <v>150</v>
+      </c>
+      <c r="C42" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>142</v>
+      </c>
+      <c r="B43" t="s">
+        <v>151</v>
+      </c>
+      <c r="C43" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s">
+        <v>142</v>
+      </c>
+      <c r="B44" t="s">
+        <v>152</v>
+      </c>
+      <c r="C44" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s">
+        <v>142</v>
+      </c>
+      <c r="B45" t="s">
+        <v>153</v>
+      </c>
+      <c r="C45" t="n">
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>